<commit_message>
updated excel files, added hough lines for each edge in square45-90 image
</commit_message>
<xml_diff>
--- a/src/square45-90_sobel_exp.bin.hough2022-02-12.xlsx
+++ b/src/square45-90_sobel_exp.bin.hough2022-02-12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F3D6D0-F2F6-4B0D-81C2-939513E69078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E196DEA6-0966-4715-BBFB-64B560C2A32C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="250" windowWidth="11300" windowHeight="8220" xr2:uid="{F57F6AC1-6941-4E32-B320-94C304BC531E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{F57F6AC1-6941-4E32-B320-94C304BC531E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="154">
+  <dxfs count="134">
     <dxf>
       <fill>
         <patternFill>
@@ -193,6 +193,48 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFCC66FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCCFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF6699"/>
         </patternFill>
       </fill>
@@ -606,6 +648,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF66FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
@@ -635,195 +684,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF66FF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF6699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF66FF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1560,28 +1420,28 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:T17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="2.6328125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="7.08984375" customWidth="1"/>
-    <col min="7" max="8" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="6.08984375" customWidth="1"/>
-    <col min="10" max="10" width="2.6328125" style="8" customWidth="1"/>
-    <col min="11" max="11" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="4.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6.453125" customWidth="1"/>
-    <col min="14" max="14" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="2.6328125" style="8" customWidth="1"/>
-    <col min="16" max="16" width="6.90625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7265625" customWidth="1"/>
-    <col min="18" max="20" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.6640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="7.109375" customWidth="1"/>
+    <col min="7" max="8" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.109375" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.44140625" customWidth="1"/>
+    <col min="14" max="14" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="2.6640625" style="8" customWidth="1"/>
+    <col min="16" max="16" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.77734375" customWidth="1"/>
+    <col min="18" max="20" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="B2" s="5">
         <v>42</v>
       </c>
@@ -1625,7 +1485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1678,7 +1538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="F4" s="5">
         <v>-8.5</v>
       </c>
@@ -1719,7 +1579,7 @@
         <v>10551</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>-157.5</v>
       </c>
@@ -1772,7 +1632,7 @@
         <v>12452</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>-156.5</v>
       </c>
@@ -1825,7 +1685,7 @@
         <v>19762</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>-155.5</v>
       </c>
@@ -1878,7 +1738,7 @@
         <v>22761</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>-154.5</v>
       </c>
@@ -1916,7 +1776,7 @@
         <v>23482</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>-153.5</v>
       </c>
@@ -1957,7 +1817,7 @@
         <v>26418</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="F10" s="5">
         <v>157.5</v>
       </c>
@@ -1971,7 +1831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>-78.5</v>
       </c>
@@ -2009,7 +1869,7 @@
         <v>24229</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>-77.5</v>
       </c>
@@ -2047,7 +1907,7 @@
         <v>24986</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>-76.5</v>
       </c>
@@ -2076,7 +1936,7 @@
         <v>27461</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>-75.5</v>
       </c>
@@ -2105,7 +1965,7 @@
         <v>23109</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>-74.5</v>
       </c>
@@ -2134,7 +1994,7 @@
         <v>16772</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>-73.5</v>
       </c>
@@ -2163,7 +2023,7 @@
         <v>11647</v>
       </c>
     </row>
-    <row r="17" spans="16:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="16:20" x14ac:dyDescent="0.3">
       <c r="P17" s="5">
         <v>6.5</v>
       </c>
@@ -2179,263 +2039,263 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A5:B8 O4:O6 M6:N6 N7 N5 E9:E12 D12:D15 J4:J6 I4:I7 E4:E7 D5:D8">
-    <cfRule type="cellIs" dxfId="153" priority="88" operator="between">
+    <cfRule type="cellIs" dxfId="133" priority="88" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="89" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="90" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="91" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="149" priority="92" operator="between">
+    <cfRule type="cellIs" dxfId="132" priority="89" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="131" priority="90" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="91" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="129" priority="92" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:E2 G2">
-    <cfRule type="cellIs" dxfId="148" priority="78" operator="between">
+    <cfRule type="cellIs" dxfId="128" priority="78" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="147" priority="79" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="146" priority="80" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="81" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="82" operator="between">
+    <cfRule type="cellIs" dxfId="127" priority="79" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="80" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="125" priority="81" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="82" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12:B15">
-    <cfRule type="cellIs" dxfId="143" priority="68" operator="between">
+    <cfRule type="cellIs" dxfId="123" priority="68" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="69" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="70" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="71" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="72" operator="between">
+    <cfRule type="cellIs" dxfId="122" priority="69" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="70" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="71" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="119" priority="72" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:G7">
-    <cfRule type="cellIs" dxfId="138" priority="58" operator="between">
+    <cfRule type="cellIs" dxfId="118" priority="58" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="59" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="60" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="61" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="134" priority="62" operator="between">
+    <cfRule type="cellIs" dxfId="117" priority="59" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="116" priority="60" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="61" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="62" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:J2 L2">
-    <cfRule type="cellIs" dxfId="133" priority="53" operator="between">
+    <cfRule type="cellIs" dxfId="113" priority="53" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="54" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="55" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="56" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="129" priority="57" operator="between">
+    <cfRule type="cellIs" dxfId="112" priority="54" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="55" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="56" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="57" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:O2">
-    <cfRule type="cellIs" dxfId="128" priority="43" operator="between">
+    <cfRule type="cellIs" dxfId="108" priority="43" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="44" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="45" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="46" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="47" operator="between">
+    <cfRule type="cellIs" dxfId="107" priority="44" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="45" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="46" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="104" priority="47" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L7">
-    <cfRule type="cellIs" dxfId="123" priority="38" operator="between">
+    <cfRule type="cellIs" dxfId="103" priority="38" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="39" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="40" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="41" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="42" operator="between">
+    <cfRule type="cellIs" dxfId="102" priority="39" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="101" priority="40" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="41" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="99" priority="42" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16 D15">
-    <cfRule type="cellIs" dxfId="118" priority="36" operator="between">
+    <cfRule type="cellIs" dxfId="98" priority="36" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P7:Q7">
-    <cfRule type="cellIs" dxfId="117" priority="32" operator="between">
+    <cfRule type="cellIs" dxfId="97" priority="32" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P6:Q6 P8:Q8">
-    <cfRule type="cellIs" dxfId="116" priority="29" operator="between">
+    <cfRule type="cellIs" dxfId="96" priority="29" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R6">
-    <cfRule type="cellIs" dxfId="115" priority="28" operator="between">
+    <cfRule type="cellIs" dxfId="95" priority="28" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q15">
-    <cfRule type="cellIs" dxfId="114" priority="25" operator="between">
+    <cfRule type="cellIs" dxfId="94" priority="25" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q14 Q16">
-    <cfRule type="cellIs" dxfId="113" priority="24" operator="between">
+    <cfRule type="cellIs" dxfId="93" priority="24" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2">
-    <cfRule type="cellIs" dxfId="112" priority="19" operator="between">
+    <cfRule type="cellIs" dxfId="92" priority="19" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="20" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="21" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="22" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="23" operator="between">
+    <cfRule type="cellIs" dxfId="91" priority="20" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="90" priority="21" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="89" priority="22" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="88" priority="23" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:I12">
-    <cfRule type="cellIs" dxfId="107" priority="14" operator="between">
+    <cfRule type="cellIs" dxfId="87" priority="14" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="15" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="16" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="17" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="18" operator="between">
+    <cfRule type="cellIs" dxfId="86" priority="15" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="85" priority="16" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="84" priority="17" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="83" priority="18" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F9:F12">
-    <cfRule type="cellIs" dxfId="102" priority="9" operator="between">
+    <cfRule type="cellIs" dxfId="82" priority="9" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="10" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="11" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="99" priority="12" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="13" operator="between">
+    <cfRule type="cellIs" dxfId="81" priority="10" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="80" priority="11" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="79" priority="12" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="78" priority="13" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q9">
-    <cfRule type="cellIs" dxfId="97" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="77" priority="1" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
@@ -2451,10 +2311,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:P29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:P27"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B2" s="5">
+        <v>174</v>
+      </c>
       <c r="C2" s="5">
         <v>177</v>
       </c>
@@ -2486,7 +2349,11 @@
         <v>138</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B3" s="6">
+        <f>B2/3</f>
+        <v>58</v>
+      </c>
       <c r="C3" s="6">
         <v>59</v>
       </c>
@@ -2525,8 +2392,8 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B4" s="5">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="5">
         <v>-159.5</v>
       </c>
       <c r="C4">
@@ -2554,8 +2421,8 @@
         <v>3442</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B5" s="5">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="5">
         <v>-160.5</v>
       </c>
       <c r="C5">
@@ -2595,8 +2462,8 @@
         <v>1821</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B6" s="5">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
         <v>-161.5</v>
       </c>
       <c r="C6">
@@ -2636,8 +2503,8 @@
         <v>2600</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B7" s="5">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="5">
         <v>-162.5</v>
       </c>
       <c r="C7">
@@ -2677,8 +2544,8 @@
         <v>2759</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B8" s="5">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="5">
         <v>-163.5</v>
       </c>
       <c r="C8">
@@ -2715,8 +2582,8 @@
         <v>3373</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B9" s="5">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="5">
         <v>-164.5</v>
       </c>
       <c r="C9">
@@ -2744,14 +2611,17 @@
         <v>2914</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B11" s="5">
-        <v>174</v>
-      </c>
-      <c r="C11" s="5">
-        <v>177</v>
-      </c>
-      <c r="D11" s="5">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" s="5">
+        <v>-8.5</v>
+      </c>
+      <c r="B11">
+        <v>22774</v>
+      </c>
+      <c r="C11">
+        <v>22264</v>
+      </c>
+      <c r="D11">
         <v>0</v>
       </c>
       <c r="H11" s="5">
@@ -2766,17 +2636,30 @@
       <c r="K11">
         <v>3401</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="B12" s="6">
-        <f>B11/3</f>
-        <v>58</v>
-      </c>
-      <c r="C12" s="6">
-        <v>59</v>
-      </c>
-      <c r="D12" s="6">
-        <f>D11/3</f>
+      <c r="M11" s="5">
+        <v>293.5</v>
+      </c>
+      <c r="N11">
+        <v>1911</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <v>-7.5</v>
+      </c>
+      <c r="B12">
+        <v>22917</v>
+      </c>
+      <c r="C12" s="10">
+        <v>40867</v>
+      </c>
+      <c r="D12">
         <v>0</v>
       </c>
       <c r="H12" s="5">
@@ -2791,16 +2674,28 @@
       <c r="K12">
         <v>2330</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M12" s="5">
+        <v>294.5</v>
+      </c>
+      <c r="N12">
+        <v>3471</v>
+      </c>
+      <c r="O12">
+        <v>23399</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
-        <v>-8.5</v>
+        <v>-6.5</v>
       </c>
       <c r="B13">
-        <v>22774</v>
-      </c>
-      <c r="C13">
-        <v>22264</v>
+        <v>26253</v>
+      </c>
+      <c r="C13" s="2">
+        <v>42912</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -2817,16 +2712,28 @@
       <c r="K13">
         <v>2754</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M13" s="5">
+        <v>295.5</v>
+      </c>
+      <c r="N13">
+        <v>2059</v>
+      </c>
+      <c r="O13">
+        <v>32551</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
-        <v>-7.5</v>
+        <v>-5.5</v>
       </c>
       <c r="B14">
-        <v>22917</v>
-      </c>
-      <c r="C14" s="10">
-        <v>40867</v>
+        <v>21037</v>
+      </c>
+      <c r="C14">
+        <v>30072</v>
       </c>
       <c r="D14">
         <v>0</v>
@@ -2843,20 +2750,20 @@
       <c r="K14">
         <v>3004</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15" s="5">
-        <v>-6.5</v>
-      </c>
-      <c r="B15">
-        <v>26253</v>
-      </c>
-      <c r="C15" s="2">
-        <v>42912</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
+      <c r="M14" s="5">
+        <v>296.5</v>
+      </c>
+      <c r="N14">
+        <v>2339</v>
+      </c>
+      <c r="O14">
+        <v>32339</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="H15" s="5">
         <v>-74.5</v>
       </c>
@@ -2869,19 +2776,31 @@
       <c r="K15">
         <v>2446</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="M15" s="5">
+        <v>297.5</v>
+      </c>
+      <c r="N15">
+        <v>3226</v>
+      </c>
+      <c r="O15">
+        <v>23227</v>
+      </c>
+      <c r="P15">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
-        <v>-5.5</v>
-      </c>
-      <c r="B16">
-        <v>21037</v>
-      </c>
-      <c r="C16">
-        <v>30072</v>
+        <v>0.5</v>
       </c>
       <c r="D16">
         <v>0</v>
+      </c>
+      <c r="E16">
+        <v>24019</v>
+      </c>
+      <c r="F16">
+        <v>24229</v>
       </c>
       <c r="H16" s="5">
         <v>-73.5</v>
@@ -2895,522 +2814,518 @@
       <c r="K16">
         <v>3203</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B18" s="5">
-        <v>0.5</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>24019</v>
+      <c r="M16" s="5">
+        <v>298.5</v>
+      </c>
+      <c r="N16">
+        <v>1811</v>
+      </c>
+      <c r="O16">
+        <v>1822</v>
+      </c>
+      <c r="P16">
+        <v>8514</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="5">
+        <v>1.5</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>30684</v>
+      </c>
+      <c r="F17">
+        <v>24986</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="5">
+        <v>2.5</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18" s="1">
+        <v>15898</v>
+      </c>
+      <c r="E18" s="3">
+        <v>47841</v>
       </c>
       <c r="F18">
-        <v>24229</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B19" s="5">
-        <v>1.5</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19">
-        <v>30684</v>
+        <v>27461</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="7">
+        <v>3.5</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19" s="2">
+        <v>77282</v>
+      </c>
+      <c r="E19" s="4">
+        <v>41900</v>
       </c>
       <c r="F19">
-        <v>24986</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B20" s="5">
-        <v>2.5</v>
+        <v>23109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="5">
+        <v>4.5</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
-      <c r="D20" s="1">
-        <v>15898</v>
-      </c>
-      <c r="E20" s="3">
-        <v>47841</v>
+      <c r="D20">
+        <v>18646</v>
+      </c>
+      <c r="E20" s="1">
+        <v>27491</v>
       </c>
       <c r="F20">
-        <v>27461</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B21" s="7">
-        <v>3.5</v>
+        <v>16772</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="5">
+        <v>5.5</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21" s="2">
-        <v>77282</v>
-      </c>
-      <c r="E21" s="4">
-        <v>41900</v>
+        <v>80299</v>
+      </c>
+      <c r="E21" s="1">
+        <v>17263</v>
       </c>
       <c r="F21">
-        <v>23109</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B22" s="5">
-        <v>4.5</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
+        <v>11647</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="5">
+        <v>6.5</v>
       </c>
       <c r="D22">
-        <v>18646</v>
-      </c>
-      <c r="E22" s="1">
-        <v>27491</v>
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>16772</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B23" s="5">
-        <v>5.5</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23" s="2">
-        <v>80299</v>
-      </c>
-      <c r="E23" s="1">
-        <v>17263</v>
-      </c>
-      <c r="F23">
-        <v>11647</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B24" s="5">
-        <v>6.5</v>
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="5">
+        <v>156.5</v>
+      </c>
+      <c r="B24">
+        <v>22404</v>
+      </c>
+      <c r="C24">
+        <v>28730</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-      <c r="F24">
-        <v>2035</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="5">
+        <v>157.5</v>
+      </c>
+      <c r="B25">
+        <v>20508</v>
+      </c>
+      <c r="C25">
+        <v>35708</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
-        <v>156.5</v>
+        <v>158.5</v>
       </c>
       <c r="B26">
-        <v>22404</v>
-      </c>
-      <c r="C26">
-        <v>28730</v>
+        <v>18277</v>
+      </c>
+      <c r="C26" s="2">
+        <v>43490</v>
       </c>
       <c r="D26">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
-        <v>157.5</v>
+        <v>159.5</v>
       </c>
       <c r="B27">
-        <v>20508</v>
+        <v>12075</v>
       </c>
       <c r="C27">
-        <v>35708</v>
+        <v>30333</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" s="5">
-        <v>158.5</v>
-      </c>
-      <c r="B28">
-        <v>18277</v>
-      </c>
-      <c r="C28" s="2">
-        <v>43490</v>
-      </c>
-      <c r="D28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>159.5</v>
-      </c>
-      <c r="B29">
-        <v>12075</v>
-      </c>
-      <c r="C29">
-        <v>30333</v>
-      </c>
-      <c r="D29">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B7:C7">
-    <cfRule type="cellIs" dxfId="96" priority="77" operator="between">
+  <conditionalFormatting sqref="C6:C8 A6:A8">
+    <cfRule type="cellIs" dxfId="76" priority="101" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:C6 B8:C8">
-    <cfRule type="cellIs" dxfId="95" priority="76" operator="between">
+  <conditionalFormatting sqref="D6">
+    <cfRule type="cellIs" dxfId="75" priority="99" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6">
-    <cfRule type="cellIs" dxfId="94" priority="75" operator="between">
+  <conditionalFormatting sqref="C2">
+    <cfRule type="cellIs" dxfId="74" priority="94" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="73" priority="95" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="72" priority="96" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="71" priority="97" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="70" priority="98" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
+    <cfRule type="cellIs" dxfId="69" priority="93" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2">
-    <cfRule type="cellIs" dxfId="93" priority="70" operator="between">
+  <conditionalFormatting sqref="D11:D14">
+    <cfRule type="cellIs" dxfId="68" priority="88" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="71" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="72" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="73" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="74" operator="between">
+    <cfRule type="cellIs" dxfId="67" priority="89" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="90" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="65" priority="91" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="92" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="cellIs" dxfId="88" priority="69" operator="between">
+  <conditionalFormatting sqref="B2">
+    <cfRule type="cellIs" dxfId="63" priority="83" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="62" priority="84" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="85" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="60" priority="86" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="59" priority="87" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A12:B14">
+    <cfRule type="cellIs" dxfId="58" priority="78" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="57" priority="79" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="80" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="81" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="82" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20">
+    <cfRule type="cellIs" dxfId="53" priority="72" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D13:D16">
-    <cfRule type="cellIs" dxfId="67" priority="64" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="65" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="66" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="67" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="68" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11">
-    <cfRule type="cellIs" dxfId="62" priority="59" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="60" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="61" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="59" priority="62" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="63" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A14:B16">
-    <cfRule type="cellIs" dxfId="57" priority="54" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="55" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="56" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="57" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="58" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11:D11">
-    <cfRule type="cellIs" dxfId="52" priority="49" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="50" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="51" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="52" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="53" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="cellIs" dxfId="47" priority="48" operator="between">
+  <conditionalFormatting sqref="C19 C21">
+    <cfRule type="cellIs" dxfId="52" priority="71" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21 C23">
-    <cfRule type="cellIs" dxfId="46" priority="47" operator="between">
+  <conditionalFormatting sqref="D24:D27">
+    <cfRule type="cellIs" dxfId="51" priority="66" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="50" priority="67" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="68" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="69" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="70" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A24:A27">
+    <cfRule type="cellIs" dxfId="46" priority="61" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="62" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="44" priority="63" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="64" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="65" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:I8 K12:K15 K5:K8">
+    <cfRule type="cellIs" dxfId="41" priority="56" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="57" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="58" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="59" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="60" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:K2">
+    <cfRule type="cellIs" dxfId="36" priority="51" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="35" priority="52" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="53" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="54" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="55" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H12:I15">
+    <cfRule type="cellIs" dxfId="31" priority="46" operator="between">
+      <formula>30000</formula>
+      <formula>40000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="47" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="48" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="49" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="50" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K15">
+    <cfRule type="cellIs" dxfId="26" priority="45" operator="between">
       <formula>80000</formula>
       <formula>111000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D26:D29">
-    <cfRule type="cellIs" dxfId="45" priority="42" operator="between">
+  <conditionalFormatting sqref="O6:P6 P7 P5">
+    <cfRule type="cellIs" dxfId="25" priority="40" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="43" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="44" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="45" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="46" operator="between">
+    <cfRule type="cellIs" dxfId="24" priority="41" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="23" priority="42" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="43" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="44" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A26:A29">
-    <cfRule type="cellIs" dxfId="40" priority="37" operator="between">
+  <conditionalFormatting sqref="N2">
+    <cfRule type="cellIs" dxfId="20" priority="35" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="38" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="39" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="40" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="41" operator="between">
+    <cfRule type="cellIs" dxfId="19" priority="36" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="37" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="38" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="39" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:I8 K12:K15 K5:K8">
-    <cfRule type="cellIs" dxfId="35" priority="32" operator="between">
+  <conditionalFormatting sqref="O2:P2">
+    <cfRule type="cellIs" dxfId="15" priority="30" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="33" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="34" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="35" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="36" operator="between">
+    <cfRule type="cellIs" dxfId="14" priority="31" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="32" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="33" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="34" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:K2">
-    <cfRule type="cellIs" dxfId="30" priority="27" operator="between">
+  <conditionalFormatting sqref="N5:N7">
+    <cfRule type="cellIs" dxfId="10" priority="25" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="28" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="29" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="30" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="31" operator="between">
+    <cfRule type="cellIs" dxfId="9" priority="26" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="27" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="28" operator="between">
+      <formula>60000</formula>
+      <formula>70000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="29" operator="between">
       <formula>70000</formula>
       <formula>100000</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H12:I15">
-    <cfRule type="cellIs" dxfId="25" priority="22" operator="between">
+  <conditionalFormatting sqref="N11:P16">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="between">
+      <formula>70000</formula>
+      <formula>100000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="between">
+      <formula>50000</formula>
+      <formula>60000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="between">
+      <formula>40000</formula>
+      <formula>50000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="between">
       <formula>30000</formula>
       <formula>40000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="23" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="25" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="26" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K15">
-    <cfRule type="cellIs" dxfId="20" priority="21" operator="between">
-      <formula>80000</formula>
-      <formula>111000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O6:P6 P7 P5">
-    <cfRule type="cellIs" dxfId="19" priority="16" operator="between">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="between">
+      <formula>20000</formula>
       <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="17" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="19" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="20" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2">
-    <cfRule type="cellIs" dxfId="14" priority="11" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="12" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="13" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="14" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="15" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O2:P2">
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="7" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="9" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="10" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N7">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="between">
-      <formula>30000</formula>
-      <formula>40000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="between">
-      <formula>40000</formula>
-      <formula>50000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="between">
-      <formula>50000</formula>
-      <formula>60000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="between">
-      <formula>60000</formula>
-      <formula>70000</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="between">
-      <formula>70000</formula>
-      <formula>100000</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="between">
+      <formula>10000</formula>
+      <formula>20000</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions gridLines="1"/>

</xml_diff>